<commit_message>
Agregar categoría Tipo (Diseñador/Árabe): nueva columna + filtros en catálogo
</commit_message>
<xml_diff>
--- a/data/catalogo.xlsx
+++ b/data/catalogo.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -570,35 +570,40 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Tamaño (ml)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Notas / Descripcion</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Precio (UYU)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Precio antes (UYU)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Promocion</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Imagen URL</t>
         </is>
@@ -623,29 +628,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Bergamota, pimienta de Sichuán, ambroxan. Fresco y especiado.</t>
         </is>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="H2" s="4" t="n">
         <v>10600</v>
       </c>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I2" s="5" t="n"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.31861.jpg</t>
         </is>
@@ -670,31 +680,36 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Cuero, canela, pomelo sangriento. Dulce y magnético.</t>
         </is>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="H3" s="8" t="n">
         <v>4590</v>
       </c>
-      <c r="H3" s="9" t="n">
+      <c r="I3" s="9" t="n">
         <v>5100</v>
       </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.3747.jpg</t>
         </is>
@@ -719,29 +734,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Gin tónic, menta, cuero vegetal. Fresco, nocturno.</t>
         </is>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="H4" s="4" t="n">
         <v>5800</v>
       </c>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I4" s="5" t="n"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.12865.jpg</t>
         </is>
@@ -766,29 +786,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E5" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>Marino, bergamota, pachulí. Fresco acuático icónico.</t>
         </is>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="H5" s="12" t="n">
         <v>7500</v>
       </c>
-      <c r="H5" s="13" t="n"/>
-      <c r="I5" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I5" s="13" t="n"/>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.410.jpg</t>
         </is>
@@ -813,29 +838,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Pomelo, laurel marino, ambergris. Deportivo y magnético.</t>
         </is>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>5200</v>
       </c>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I6" s="5" t="n"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.18471.jpg</t>
         </is>
@@ -860,29 +890,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E7" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>Bergamota, pimienta, lavanda, vainilla ambarada. Más profundo que el EDT.</t>
         </is>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="H7" s="12" t="n">
         <v>12500</v>
       </c>
-      <c r="H7" s="13" t="n"/>
-      <c r="I7" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I7" s="13" t="n"/>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L7" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.48100.jpg</t>
         </is>
@@ -907,29 +942,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Iris polvoriento, lavanda, ámbar, pera. Masculino, elegante, invernal.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="H8" s="4" t="n">
         <v>12800</v>
       </c>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I8" s="5" t="n"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.13016.jpg</t>
         </is>
@@ -954,29 +994,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E9" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>Iris, salvia, vetiver. Fresco, refinado y misterioso.</t>
         </is>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="H9" s="12" t="n">
         <v>12000</v>
       </c>
-      <c r="H9" s="13" t="n"/>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I9" s="13" t="n"/>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.13015.jpg</t>
         </is>
@@ -1001,29 +1046,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Espino, madreselva, violeta, cuero. Clásico atemporal.</t>
         </is>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>9200</v>
       </c>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I10" s="5" t="n"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.384.jpg</t>
         </is>
@@ -1048,29 +1098,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E11" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>Limón, albahaca, romero. Cítrico aromático clásico.</t>
         </is>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="H11" s="12" t="n">
         <v>8400</v>
       </c>
-      <c r="H11" s="13" t="n"/>
-      <c r="I11" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I11" s="13" t="n"/>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K11" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L11" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.231.jpg</t>
         </is>
@@ -1095,29 +1150,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Lavanda, limón, cardamomo, vetiver. Fresco tecno-moderno.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>5900</v>
       </c>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I12" s="5" t="n"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.68226.jpg</t>
         </is>
@@ -1142,29 +1202,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E13" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>Tomillo, jengibre, canela, cuero. Oriental especiado sensual.</t>
         </is>
       </c>
-      <c r="G13" s="12" t="n">
+      <c r="H13" s="12" t="n">
         <v>5400</v>
       </c>
-      <c r="H13" s="13" t="n"/>
-      <c r="I13" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I13" s="13" t="n"/>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K13" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.46038.jpg</t>
         </is>
@@ -1189,29 +1254,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Mandarina sanguina, cardamomo, cuero ambarado. Más intenso que el EDT.</t>
         </is>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>5800</v>
       </c>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I14" s="5" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.60035.jpg</t>
         </is>
@@ -1236,29 +1306,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E15" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F15" s="11" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>Olíbano, caoba, pachulí. Seductor, oriental especiado.</t>
         </is>
       </c>
-      <c r="G15" s="12" t="n">
+      <c r="H15" s="12" t="n">
         <v>6200</v>
       </c>
-      <c r="H15" s="13" t="n"/>
-      <c r="I15" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I15" s="13" t="n"/>
       <c r="J15" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K15" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L15" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.78575.jpg</t>
         </is>
@@ -1283,29 +1358,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Laurel, jazmín, ambroxan. Acuático aromático intensificado.</t>
         </is>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="H16" s="4" t="n">
         <v>5900</v>
       </c>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I16" s="5" t="n"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.90433.jpg</t>
         </is>
@@ -1330,29 +1410,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E17" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F17" s="11" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
         <is>
           <t>Bergamota, pimienta verde, incienso, gengibre. Fresco urbano.</t>
         </is>
       </c>
-      <c r="G17" s="12" t="n">
+      <c r="H17" s="12" t="n">
         <v>5400</v>
       </c>
-      <c r="H17" s="13" t="n"/>
-      <c r="I17" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I17" s="13" t="n"/>
       <c r="J17" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K17" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.297.jpg</t>
         </is>
@@ -1377,29 +1462,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Menta, ron, cuero, regaliz. Intenso, nocturno, dulce.</t>
         </is>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="H18" s="4" t="n">
         <v>6200</v>
       </c>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I18" s="5" t="n"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.46093.jpg</t>
         </is>
@@ -1424,29 +1514,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E19" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F19" s="11" t="inlineStr">
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
         <is>
           <t>Pimienta blanca, salvia, cacao, tonka. Amargo gourmand moderno.</t>
         </is>
       </c>
-      <c r="G19" s="12" t="n">
+      <c r="H19" s="12" t="n">
         <v>6800</v>
       </c>
-      <c r="H19" s="13" t="n"/>
-      <c r="I19" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I19" s="13" t="n"/>
       <c r="J19" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K19" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L19" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.55449.jpg</t>
         </is>
@@ -1471,29 +1566,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Pimienta, sabio, plum, cedro, vainilla. Más frutal e intenso.</t>
         </is>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="H20" s="4" t="n">
         <v>7500</v>
       </c>
-      <c r="H20" s="5" t="n"/>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I20" s="5" t="n"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.71888.jpg</t>
         </is>
@@ -1518,29 +1618,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E21" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
         <is>
           <t>Pomelo, lavanda, canela, cuero. Elegante, sofisticado.</t>
         </is>
       </c>
-      <c r="G21" s="12" t="n">
+      <c r="H21" s="12" t="n">
         <v>5600</v>
       </c>
-      <c r="H21" s="13" t="n"/>
-      <c r="I21" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I21" s="13" t="n"/>
       <c r="J21" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K21" s="11" t="inlineStr"/>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K21" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L21" s="11" t="inlineStr"/>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="2" t="n">
@@ -1561,29 +1666,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E22" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Incienso, salvia, menta, pachulí. Versión más intensa del Giò.</t>
         </is>
       </c>
-      <c r="G22" s="4" t="n">
+      <c r="H22" s="4" t="n">
         <v>9800</v>
       </c>
-      <c r="H22" s="5" t="n"/>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I22" s="5" t="n"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.29727.jpg</t>
         </is>
@@ -1608,29 +1718,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E23" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
         <is>
           <t>Vetiver, pachulí, incienso. Intensísimo, recargable.</t>
         </is>
       </c>
-      <c r="G23" s="12" t="n">
+      <c r="H23" s="12" t="n">
         <v>11200</v>
       </c>
-      <c r="H23" s="13" t="n"/>
-      <c r="I23" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I23" s="13" t="n"/>
       <c r="J23" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K23" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L23" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.81508.jpg</t>
         </is>
@@ -1655,29 +1770,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Anís estrellado, limón, oliva, tonka. Oriental aromático dulce.</t>
         </is>
       </c>
-      <c r="G24" s="4" t="n">
+      <c r="H24" s="4" t="n">
         <v>7800</v>
       </c>
-      <c r="H24" s="5" t="n"/>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I24" s="5" t="n"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.412.jpg</t>
         </is>
@@ -1702,29 +1822,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E25" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F25" s="11" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
         <is>
           <t>Castaña, menta, salvia, vainilla, smoke. Dulce gourmand moderno.</t>
         </is>
       </c>
-      <c r="G25" s="12" t="n">
+      <c r="H25" s="12" t="n">
         <v>6800</v>
       </c>
-      <c r="H25" s="13" t="n"/>
-      <c r="I25" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I25" s="13" t="n"/>
       <c r="J25" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K25" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K25" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L25" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.45258.jpg</t>
         </is>
@@ -1749,29 +1874,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E26" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Manzana, canela, clavo, sándalo. Clásico masculino universal.</t>
         </is>
       </c>
-      <c r="G26" s="4" t="n">
+      <c r="H26" s="4" t="n">
         <v>5200</v>
       </c>
-      <c r="H26" s="5" t="n"/>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I26" s="5" t="n"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K26" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.383.jpg</t>
         </is>
@@ -1796,29 +1926,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E27" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F27" s="11" t="inlineStr">
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
         <is>
           <t>Canela, manzana, cuero, cedro. Intensificado, más persistente.</t>
         </is>
       </c>
-      <c r="G27" s="12" t="n">
+      <c r="H27" s="12" t="n">
         <v>7500</v>
       </c>
-      <c r="H27" s="13" t="n"/>
-      <c r="I27" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I27" s="13" t="n"/>
       <c r="J27" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K27" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K27" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L27" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.75183.jpg</t>
         </is>
@@ -1843,29 +1978,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E28" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Mandarina, maninka, cuero. Seductor especiado.</t>
         </is>
       </c>
-      <c r="G28" s="4" t="n">
+      <c r="H28" s="4" t="n">
         <v>5800</v>
       </c>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I28" s="5" t="n"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K28" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.31445.jpg</t>
         </is>
@@ -1890,29 +2030,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E29" s="10" t="n">
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="F29" s="11" t="inlineStr">
+      <c r="G29" s="11" t="inlineStr">
         <is>
           <t>Menta, manzana verde, lavanda, abeto. Fresco juvenil icónico.</t>
         </is>
       </c>
-      <c r="G29" s="12" t="n">
+      <c r="H29" s="12" t="n">
         <v>4200</v>
       </c>
-      <c r="H29" s="13" t="n"/>
-      <c r="I29" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I29" s="13" t="n"/>
       <c r="J29" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K29" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K29" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L29" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.570.jpg</t>
         </is>
@@ -1937,29 +2082,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E30" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Pomelo, cardamomo, romero, cedro. Limpio y fresco.</t>
         </is>
       </c>
-      <c r="G30" s="4" t="n">
+      <c r="H30" s="4" t="n">
         <v>4800</v>
       </c>
-      <c r="H30" s="5" t="n"/>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I30" s="5" t="n"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K30" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.11043.jpg</t>
         </is>
@@ -1984,29 +2134,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E31" s="10" t="n">
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="F31" s="11" t="inlineStr">
+      <c r="G31" s="11" t="inlineStr">
         <is>
           <t>Uva, pepino, vetiver, cedro. Verde fresco deportivo.</t>
         </is>
       </c>
-      <c r="G31" s="12" t="n">
+      <c r="H31" s="12" t="n">
         <v>4500</v>
       </c>
-      <c r="H31" s="13" t="n"/>
-      <c r="I31" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I31" s="13" t="n"/>
       <c r="J31" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K31" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K31" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L31" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.787.jpg</t>
         </is>
@@ -2031,29 +2186,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E32" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Lavanda, geranio, cedro, sándalo. Aromático clásico noventero.</t>
         </is>
       </c>
-      <c r="G32" s="4" t="n">
+      <c r="H32" s="4" t="n">
         <v>5200</v>
       </c>
-      <c r="H32" s="5" t="n"/>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I32" s="5" t="n"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K32" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.258.jpg</t>
         </is>
@@ -2078,29 +2238,34 @@
           <t>Unisex</t>
         </is>
       </c>
-      <c r="E33" s="10" t="n">
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="n">
         <v>200</v>
       </c>
-      <c r="F33" s="11" t="inlineStr">
+      <c r="G33" s="11" t="inlineStr">
         <is>
           <t>Limón, bergamota, papaya, té verde. Unisex fresco icónico.</t>
         </is>
       </c>
-      <c r="G33" s="12" t="n">
+      <c r="H33" s="12" t="n">
         <v>4200</v>
       </c>
-      <c r="H33" s="13" t="n"/>
-      <c r="I33" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I33" s="13" t="n"/>
       <c r="J33" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K33" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K33" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L33" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.276.jpg</t>
         </is>
@@ -2125,29 +2290,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n">
         <v>125</v>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Mandarina, lavanda, amberes, almizcle. Oriental especiado 80s.</t>
         </is>
       </c>
-      <c r="G34" s="4" t="n">
+      <c r="H34" s="4" t="n">
         <v>4600</v>
       </c>
-      <c r="H34" s="5" t="n"/>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I34" s="5" t="n"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.251.jpg</t>
         </is>
@@ -2172,29 +2342,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E35" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F35" s="11" t="inlineStr">
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
         <is>
           <t>Menta, manzana verde, tonka, vainilla, vetiver. Dulce aromático icónico.</t>
         </is>
       </c>
-      <c r="G35" s="12" t="n">
+      <c r="H35" s="12" t="n">
         <v>6500</v>
       </c>
-      <c r="H35" s="13" t="n"/>
-      <c r="I35" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I35" s="13" t="n"/>
       <c r="J35" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K35" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K35" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L35" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.16657.jpg</t>
         </is>
@@ -2219,29 +2394,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E36" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>Menta, manzana, madera, vainilla cremosa. Más oriental que el EDT.</t>
         </is>
       </c>
-      <c r="G36" s="4" t="n">
+      <c r="H36" s="4" t="n">
         <v>7200</v>
       </c>
-      <c r="H36" s="5" t="n"/>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I36" s="5" t="n"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K36" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.62762.jpg</t>
         </is>
@@ -2266,29 +2446,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E37" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F37" s="11" t="inlineStr">
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
         <is>
           <t>Bergamota, pomelo, pimienta rosa, pachulí. Moderno fresco.</t>
         </is>
       </c>
-      <c r="G37" s="12" t="n">
+      <c r="H37" s="12" t="n">
         <v>6200</v>
       </c>
-      <c r="H37" s="13" t="n"/>
-      <c r="I37" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I37" s="13" t="n"/>
       <c r="J37" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K37" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K37" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L37" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.40031.jpg</t>
         </is>
@@ -2313,29 +2498,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E38" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>Bergamota, neroli, clary sage, cedro. Fresco aromático mediterráneo.</t>
         </is>
       </c>
-      <c r="G38" s="4" t="n">
+      <c r="H38" s="4" t="n">
         <v>5800</v>
       </c>
-      <c r="H38" s="5" t="n"/>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I38" s="5" t="n"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K38" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.2318.jpg</t>
         </is>
@@ -2360,29 +2550,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E39" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F39" s="11" t="inlineStr">
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
         <is>
           <t>Limón, pimienta, cardamomo, cuero, vetiver. Especiado carismático.</t>
         </is>
       </c>
-      <c r="G39" s="12" t="n">
+      <c r="H39" s="12" t="n">
         <v>5800</v>
       </c>
-      <c r="H39" s="13" t="n"/>
-      <c r="I39" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I39" s="13" t="n"/>
       <c r="J39" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K39" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K39" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L39" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.38686.jpg</t>
         </is>
@@ -2407,29 +2602,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E40" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
         <is>
           <t>Limón, bergamota, jazmín, almizcle. Fresco acuático.</t>
         </is>
       </c>
-      <c r="G40" s="4" t="n">
+      <c r="H40" s="4" t="n">
         <v>5200</v>
       </c>
-      <c r="H40" s="5" t="n"/>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I40" s="5" t="n"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K40" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.788.jpg</t>
         </is>
@@ -2454,29 +2654,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E41" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F41" s="11" t="inlineStr">
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F41" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
         <is>
           <t>Lavanda, manzana, menta, cuero. Fresco americano casual.</t>
         </is>
       </c>
-      <c r="G41" s="12" t="n">
+      <c r="H41" s="12" t="n">
         <v>4500</v>
       </c>
-      <c r="H41" s="13" t="n"/>
-      <c r="I41" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I41" s="13" t="n"/>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K41" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K41" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L41" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.6314.jpg</t>
         </is>
@@ -2501,29 +2706,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
         <is>
           <t>Manzana, loto, abeto, musgo. Acuático aromático fresco.</t>
         </is>
       </c>
-      <c r="G42" s="4" t="n">
+      <c r="H42" s="4" t="n">
         <v>3800</v>
       </c>
-      <c r="H42" s="5" t="n"/>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I42" s="5" t="n"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K42" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.913.jpg</t>
         </is>
@@ -2548,29 +2758,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E43" s="10" t="n">
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="F43" s="11" t="inlineStr">
+      <c r="G43" s="11" t="inlineStr">
         <is>
           <t>Lavanda, menta, cardamomo, vainilla tonka. Oriental aromático icónico.</t>
         </is>
       </c>
-      <c r="G43" s="12" t="n">
+      <c r="H43" s="12" t="n">
         <v>6500</v>
       </c>
-      <c r="H43" s="13" t="n"/>
-      <c r="I43" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I43" s="13" t="n"/>
       <c r="J43" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K43" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K43" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L43" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.430.jpg</t>
         </is>
@@ -2595,29 +2810,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E44" s="2" t="n">
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
         <v>125</v>
       </c>
-      <c r="F44" s="3" t="inlineStr">
+      <c r="G44" s="3" t="inlineStr">
         <is>
           <t>Pera negra, lavanda, canela, vainilla ámbar. Más dulce e intenso.</t>
         </is>
       </c>
-      <c r="G44" s="4" t="n">
+      <c r="H44" s="4" t="n">
         <v>7200</v>
       </c>
-      <c r="H44" s="5" t="n"/>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I44" s="5" t="n"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K44" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.30947.jpg</t>
         </is>
@@ -2642,29 +2862,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E45" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F45" s="11" t="inlineStr">
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F45" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
         <is>
           <t>Manzana, jengibre, salvia, ambroxan. Fresco amaderado moderno.</t>
         </is>
       </c>
-      <c r="G45" s="12" t="n">
+      <c r="H45" s="12" t="n">
         <v>8200</v>
       </c>
-      <c r="H45" s="13" t="n"/>
-      <c r="I45" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I45" s="13" t="n"/>
       <c r="J45" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K45" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K45" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L45" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.50757.jpg</t>
         </is>
@@ -2689,29 +2914,34 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E46" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F46" s="3" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
         <is>
           <t>Jengibre, bergamota, cedro, tonka. Elegante masculino.</t>
         </is>
       </c>
-      <c r="G46" s="4" t="n">
+      <c r="H46" s="4" t="n">
         <v>7800</v>
       </c>
-      <c r="H46" s="5" t="n"/>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I46" s="5" t="n"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K46" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.734.jpg</t>
         </is>
@@ -2736,29 +2966,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E47" s="10" t="n">
+      <c r="E47" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F47" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="F47" s="11" t="inlineStr">
+      <c r="G47" s="11" t="inlineStr">
         <is>
           <t>Jazmín, almendra, cacao, tonka. Floral dulce elegante.</t>
         </is>
       </c>
-      <c r="G47" s="12" t="n">
+      <c r="H47" s="12" t="n">
         <v>6800</v>
       </c>
-      <c r="H47" s="13" t="n"/>
-      <c r="I47" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I47" s="13" t="n"/>
       <c r="J47" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K47" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K47" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L47" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.39681.jpg</t>
         </is>
@@ -2783,29 +3018,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E48" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F48" s="3" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
         <is>
           <t>Iris, pera, pachulí, vainilla. Gourmand luminoso.</t>
         </is>
       </c>
-      <c r="G48" s="4" t="n">
+      <c r="H48" s="4" t="n">
         <v>8200</v>
       </c>
-      <c r="H48" s="5" t="n"/>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I48" s="5" t="n"/>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K48" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.14982.jpg</t>
         </is>
@@ -2830,29 +3070,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E49" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F49" s="11" t="inlineStr">
+      <c r="E49" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F49" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
         <is>
           <t>Rosa, jazmín, pachulí, vetiver. Oriental chic atemporal.</t>
         </is>
       </c>
-      <c r="G49" s="12" t="n">
+      <c r="H49" s="12" t="n">
         <v>10500</v>
       </c>
-      <c r="H49" s="13" t="n"/>
-      <c r="I49" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I49" s="13" t="n"/>
       <c r="J49" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K49" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K49" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L49" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.611.jpg</t>
         </is>
@@ -2877,29 +3122,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E50" s="2" t="n">
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="F50" s="3" t="inlineStr">
+      <c r="G50" s="3" t="inlineStr">
         <is>
           <t>Lavanda, azahar, vainilla madagascar. Floral sensual moderno.</t>
         </is>
       </c>
-      <c r="G50" s="4" t="n">
+      <c r="H50" s="4" t="n">
         <v>9200</v>
       </c>
-      <c r="H50" s="5" t="n"/>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I50" s="5" t="n"/>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K50" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L50" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.56077.jpg</t>
         </is>
@@ -2924,31 +3174,36 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E51" s="6" t="n">
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>80</v>
       </c>
-      <c r="F51" s="7" t="inlineStr">
+      <c r="G51" s="7" t="inlineStr">
         <is>
           <t>Champagne rosé, frutos rojos, musgo blanco. Festivo y femenino.</t>
         </is>
       </c>
-      <c r="G51" s="8" t="n">
+      <c r="H51" s="8" t="n">
         <v>5850</v>
       </c>
-      <c r="H51" s="9" t="n">
+      <c r="I51" s="9" t="n">
         <v>6500</v>
       </c>
-      <c r="I51" s="6" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="K51" s="7" t="inlineStr">
+      <c r="K51" s="6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="L51" s="7" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.22857.jpg</t>
         </is>
@@ -2973,29 +3228,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E52" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
         <is>
           <t>Pimienta rosa, jazmín, pachulí, vetiver. Fresco sofisticado.</t>
         </is>
       </c>
-      <c r="G52" s="4" t="n">
+      <c r="H52" s="4" t="n">
         <v>10800</v>
       </c>
-      <c r="H52" s="5" t="n"/>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I52" s="5" t="n"/>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K52" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.610.jpg</t>
         </is>
@@ -3020,29 +3280,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E53" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F53" s="11" t="inlineStr">
+      <c r="E53" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F53" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G53" s="11" t="inlineStr">
         <is>
           <t>Pomelo, membrillo, jazmín, iris. Frutal floral luminoso.</t>
         </is>
       </c>
-      <c r="G53" s="12" t="n">
+      <c r="H53" s="12" t="n">
         <v>10500</v>
       </c>
-      <c r="H53" s="13" t="n"/>
-      <c r="I53" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I53" s="13" t="n"/>
       <c r="J53" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K53" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K53" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L53" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.8069.jpg</t>
         </is>
@@ -3067,29 +3332,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E54" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>Pimienta, jazmín, rosa, pachulí, amber. Más denso y oriental.</t>
         </is>
       </c>
-      <c r="G54" s="4" t="n">
+      <c r="H54" s="4" t="n">
         <v>11500</v>
       </c>
-      <c r="H54" s="5" t="n"/>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I54" s="5" t="n"/>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K54" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.31351.jpg</t>
         </is>
@@ -3114,29 +3384,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E55" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F55" s="11" t="inlineStr">
+      <c r="E55" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F55" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G55" s="11" t="inlineStr">
         <is>
           <t>Aldehídos, ylang-ylang, rosa mayo, jazmín, vainilla, sándalo. Legendario.</t>
         </is>
       </c>
-      <c r="G55" s="12" t="n">
+      <c r="H55" s="12" t="n">
         <v>12500</v>
       </c>
-      <c r="H55" s="13" t="n"/>
-      <c r="I55" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I55" s="13" t="n"/>
       <c r="J55" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K55" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K55" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L55" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.40069.jpg</t>
         </is>
@@ -3161,29 +3436,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E56" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>Bergamota, rosa, jazmín, pachulí, tonka. Oriental profundo nocturno.</t>
         </is>
       </c>
-      <c r="G56" s="4" t="n">
+      <c r="H56" s="4" t="n">
         <v>11000</v>
       </c>
-      <c r="H56" s="5" t="n"/>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I56" s="5" t="n"/>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K56" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.15963.jpg</t>
         </is>
@@ -3208,29 +3488,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E57" s="10" t="n">
+      <c r="E57" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F57" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="F57" s="11" t="inlineStr">
+      <c r="G57" s="11" t="inlineStr">
         <is>
           <t>Pera, bergamota, rosa, jazmín, almizcle blanco. Floral chypre ligero.</t>
         </is>
       </c>
-      <c r="G57" s="12" t="n">
+      <c r="H57" s="12" t="n">
         <v>8500</v>
       </c>
-      <c r="H57" s="13" t="n"/>
-      <c r="I57" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I57" s="13" t="n"/>
       <c r="J57" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K57" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K57" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L57" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.55795.jpg</t>
         </is>
@@ -3255,29 +3540,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E58" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>Jengibre, pimienta, lychee, magnolia, jazmín, almizcle. Fresco floral.</t>
         </is>
       </c>
-      <c r="G58" s="4" t="n">
+      <c r="H58" s="4" t="n">
         <v>7800</v>
       </c>
-      <c r="H58" s="5" t="n"/>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I58" s="5" t="n"/>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K58" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.184.jpg</t>
         </is>
@@ -3302,29 +3592,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E59" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F59" s="11" t="inlineStr">
+      <c r="E59" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F59" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G59" s="11" t="inlineStr">
         <is>
           <t>Iris, pera, jazmín, vainilla, pachulí. Más intenso que el original.</t>
         </is>
       </c>
-      <c r="G59" s="12" t="n">
+      <c r="H59" s="12" t="n">
         <v>9800</v>
       </c>
-      <c r="H59" s="13" t="n"/>
-      <c r="I59" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I59" s="13" t="n"/>
       <c r="J59" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K59" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K59" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L59" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.59326.jpg</t>
         </is>
@@ -3349,29 +3644,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E60" s="2" t="n">
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Frutos rojos, jazmín egipcio, tonka, vetiver. Más gourmet y oscuro.</t>
         </is>
       </c>
-      <c r="G60" s="4" t="n">
+      <c r="H60" s="4" t="n">
         <v>7500</v>
       </c>
-      <c r="H60" s="5" t="n"/>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I60" s="5" t="n"/>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K60" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L60" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.61769.jpg</t>
         </is>
@@ -3396,29 +3696,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E61" s="10" t="n">
+      <c r="E61" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F61" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="F61" s="11" t="inlineStr">
+      <c r="G61" s="11" t="inlineStr">
         <is>
           <t>Grosella negra, rosa, jazmín, cacao. Rojo sensual, gourmand floral.</t>
         </is>
       </c>
-      <c r="G61" s="12" t="n">
+      <c r="H61" s="12" t="n">
         <v>7800</v>
       </c>
-      <c r="H61" s="13" t="n"/>
-      <c r="I61" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I61" s="13" t="n"/>
       <c r="J61" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K61" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K61" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L61" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.65560.jpg</t>
         </is>
@@ -3443,29 +3748,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E62" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F62" s="3" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
         <is>
           <t>Pomelo, bergamota, rosa, ámbar, cuero. Elegante clásico.</t>
         </is>
       </c>
-      <c r="G62" s="4" t="n">
+      <c r="H62" s="4" t="n">
         <v>5800</v>
       </c>
-      <c r="H62" s="5" t="n"/>
-      <c r="I62" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I62" s="5" t="n"/>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K62" s="3" t="inlineStr"/>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr"/>
     </row>
     <row r="63" ht="40" customHeight="1">
       <c r="A63" s="10" t="n">
@@ -3486,29 +3796,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E63" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F63" s="11" t="inlineStr">
+      <c r="E63" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F63" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G63" s="11" t="inlineStr">
         <is>
           <t>Mandarina, flor de loto, bambú, sándalo. Fresco urbano limpio.</t>
         </is>
       </c>
-      <c r="G63" s="12" t="n">
+      <c r="H63" s="12" t="n">
         <v>5500</v>
       </c>
-      <c r="H63" s="13" t="n"/>
-      <c r="I63" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I63" s="13" t="n"/>
       <c r="J63" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K63" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K63" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L63" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.296.jpg</t>
         </is>
@@ -3533,29 +3848,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E64" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>Pimienta rosa, gardenia, vainilla, musgo. Oriental floral sensual.</t>
         </is>
       </c>
-      <c r="G64" s="4" t="n">
+      <c r="H64" s="4" t="n">
         <v>5800</v>
       </c>
-      <c r="H64" s="5" t="n"/>
-      <c r="I64" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I64" s="5" t="n"/>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K64" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L64" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.306.jpg</t>
         </is>
@@ -3580,29 +3900,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E65" s="10" t="n">
+      <c r="E65" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F65" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="F65" s="11" t="inlineStr">
+      <c r="G65" s="11" t="inlineStr">
         <is>
           <t>Lavanda, azahar, vainilla, ámbar negro. Más oscuro y nocturno.</t>
         </is>
       </c>
-      <c r="G65" s="12" t="n">
+      <c r="H65" s="12" t="n">
         <v>10200</v>
       </c>
-      <c r="H65" s="13" t="n"/>
-      <c r="I65" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I65" s="13" t="n"/>
       <c r="J65" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K65" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K65" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L65" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.62318.jpg</t>
         </is>
@@ -3627,29 +3952,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E66" s="2" t="n">
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="F66" s="3" t="inlineStr">
+      <c r="G66" s="3" t="inlineStr">
         <is>
           <t>Café, jazmín sambac, vainilla, praliné. Oriental gourmand adictivo.</t>
         </is>
       </c>
-      <c r="G66" s="4" t="n">
+      <c r="H66" s="4" t="n">
         <v>9500</v>
       </c>
-      <c r="H66" s="5" t="n"/>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I66" s="5" t="n"/>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K66" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.25324.jpg</t>
         </is>
@@ -3674,29 +4004,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E67" s="10" t="n">
+      <c r="E67" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F67" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="F67" s="11" t="inlineStr">
+      <c r="G67" s="11" t="inlineStr">
         <is>
           <t>Fresa, pera, peonía, jazmín, pachulí. Floral frutal chypre moderno.</t>
         </is>
       </c>
-      <c r="G67" s="12" t="n">
+      <c r="H67" s="12" t="n">
         <v>9200</v>
       </c>
-      <c r="H67" s="13" t="n"/>
-      <c r="I67" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I67" s="13" t="n"/>
       <c r="J67" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K67" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K67" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L67" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.38914.jpg</t>
         </is>
@@ -3721,29 +4056,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E68" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F68" s="3" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
         <is>
           <t>Pera, magnolia, jazmín sambac, rosa, vainilla. Floral icónico luminoso.</t>
         </is>
       </c>
-      <c r="G68" s="4" t="n">
+      <c r="H68" s="4" t="n">
         <v>12500</v>
       </c>
-      <c r="H68" s="5" t="n"/>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I68" s="5" t="n"/>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K68" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.210.jpg</t>
         </is>
@@ -3768,29 +4108,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E69" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F69" s="11" t="inlineStr">
+      <c r="E69" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F69" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G69" s="11" t="inlineStr">
         <is>
           <t>Rosa grasse, lily of the valley, pachulí. Floral romántico moderno.</t>
         </is>
       </c>
-      <c r="G69" s="12" t="n">
+      <c r="H69" s="12" t="n">
         <v>11500</v>
       </c>
-      <c r="H69" s="13" t="n"/>
-      <c r="I69" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I69" s="13" t="n"/>
       <c r="J69" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K69" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K69" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L69" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.45202.jpg</t>
         </is>
@@ -3815,29 +4160,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E70" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F70" s="3" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
         <is>
           <t>Pomelo, rosa damascena, almendra amarga, vainilla. Oriental frutal.</t>
         </is>
       </c>
-      <c r="G70" s="4" t="n">
+      <c r="H70" s="4" t="n">
         <v>10500</v>
       </c>
-      <c r="H70" s="5" t="n"/>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I70" s="5" t="n"/>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K70" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L70" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.35561.jpg</t>
         </is>
@@ -3862,29 +4212,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E71" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F71" s="11" t="inlineStr">
+      <c r="E71" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F71" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G71" s="11" t="inlineStr">
         <is>
           <t>Cassis, rosa de mayo, vainilla, pachulí. Chypre moderno frutal.</t>
         </is>
       </c>
-      <c r="G71" s="12" t="n">
+      <c r="H71" s="12" t="n">
         <v>10200</v>
       </c>
-      <c r="H71" s="13" t="n"/>
-      <c r="I71" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I71" s="13" t="n"/>
       <c r="J71" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K71" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K71" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L71" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.18453.jpg</t>
         </is>
@@ -3909,29 +4264,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E72" s="2" t="n">
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="F72" s="3" t="inlineStr">
+      <c r="G72" s="3" t="inlineStr">
         <is>
           <t>Bergamota, azahar, tuberosa, vainilla, cedro blanco. Floral moderno.</t>
         </is>
       </c>
-      <c r="G72" s="4" t="n">
+      <c r="H72" s="4" t="n">
         <v>9200</v>
       </c>
-      <c r="H72" s="5" t="n"/>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I72" s="5" t="n"/>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K72" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L72" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.62036.jpg</t>
         </is>
@@ -3956,29 +4316,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E73" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F73" s="11" t="inlineStr">
+      <c r="E73" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F73" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G73" s="11" t="inlineStr">
         <is>
           <t>Pera, cassis, rosa, frangipani, vainilla. Más dulce y pasional que Sì.</t>
         </is>
       </c>
-      <c r="G73" s="12" t="n">
+      <c r="H73" s="12" t="n">
         <v>9800</v>
       </c>
-      <c r="H73" s="13" t="n"/>
-      <c r="I73" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I73" s="13" t="n"/>
       <c r="J73" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K73" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K73" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L73" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.48002.jpg</t>
         </is>
@@ -4003,29 +4368,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E74" s="2" t="n">
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="F74" s="3" t="inlineStr">
+      <c r="G74" s="3" t="inlineStr">
         <is>
           <t>Frambuesa, neroli, jazmín, naranjo, miel, pachulí. Dorado y divertido.</t>
         </is>
       </c>
-      <c r="G74" s="4" t="n">
+      <c r="H74" s="4" t="n">
         <v>6500</v>
       </c>
-      <c r="H74" s="5" t="n"/>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I74" s="5" t="n"/>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K74" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L74" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.9045.jpg</t>
         </is>
@@ -4050,29 +4420,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E75" s="10" t="n">
+      <c r="E75" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F75" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="F75" s="11" t="inlineStr">
+      <c r="G75" s="11" t="inlineStr">
         <is>
           <t>Jazmín acuático, mandarina verde, vainilla salada, sándalo. Solar sexy.</t>
         </is>
       </c>
-      <c r="G75" s="12" t="n">
+      <c r="H75" s="12" t="n">
         <v>6200</v>
       </c>
-      <c r="H75" s="13" t="n"/>
-      <c r="I75" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I75" s="13" t="n"/>
       <c r="J75" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K75" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K75" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L75" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.31666.jpg</t>
         </is>
@@ -4097,29 +4472,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E76" s="2" t="n">
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="F76" s="3" t="inlineStr">
+      <c r="G76" s="3" t="inlineStr">
         <is>
           <t>Mango, bergamota, jazmín, olíbano, vainilla, sándalo. Mineral floral.</t>
         </is>
       </c>
-      <c r="G76" s="4" t="n">
+      <c r="H76" s="4" t="n">
         <v>6800</v>
       </c>
-      <c r="H76" s="5" t="n"/>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I76" s="5" t="n"/>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K76" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L76" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.74962.jpg</t>
         </is>
@@ -4144,29 +4524,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E77" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F77" s="11" t="inlineStr">
+      <c r="E77" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F77" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G77" s="11" t="inlineStr">
         <is>
           <t>Pomelo, granada, flor loto, orquídea, amber, cream accord. Oriental seductor.</t>
         </is>
       </c>
-      <c r="G77" s="12" t="n">
+      <c r="H77" s="12" t="n">
         <v>6500</v>
       </c>
-      <c r="H77" s="13" t="n"/>
-      <c r="I77" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I77" s="13" t="n"/>
       <c r="J77" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K77" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K77" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L77" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.253.jpg</t>
         </is>
@@ -4191,29 +4576,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E78" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F78" s="3" t="inlineStr">
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
         <is>
           <t>Freesia, clavel, madreselva, sándalo. Floral clásico.</t>
         </is>
       </c>
-      <c r="G78" s="4" t="n">
+      <c r="H78" s="4" t="n">
         <v>5800</v>
       </c>
-      <c r="H78" s="5" t="n"/>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I78" s="5" t="n"/>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K78" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L78" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.257.jpg</t>
         </is>
@@ -4238,29 +4628,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E79" s="10" t="n">
+      <c r="E79" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F79" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="F79" s="11" t="inlineStr">
+      <c r="G79" s="11" t="inlineStr">
         <is>
           <t>Yuzu, granada, magnolia, peonía, lotus, almizcle. Floral acuático.</t>
         </is>
       </c>
-      <c r="G79" s="12" t="n">
+      <c r="H79" s="12" t="n">
         <v>6200</v>
       </c>
-      <c r="H79" s="13" t="n"/>
-      <c r="I79" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I79" s="13" t="n"/>
       <c r="J79" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K79" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K79" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L79" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.632.jpg</t>
         </is>
@@ -4285,29 +4680,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E80" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F80" s="3" t="inlineStr">
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
         <is>
           <t>Limón, mandarina, peonía, jazmín, ámbar, sándalo. Floral oriental.</t>
         </is>
       </c>
-      <c r="G80" s="4" t="n">
+      <c r="H80" s="4" t="n">
         <v>6800</v>
       </c>
-      <c r="H80" s="5" t="n"/>
-      <c r="I80" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I80" s="5" t="n"/>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K80" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L80" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.28958.jpg</t>
         </is>
@@ -4332,29 +4732,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E81" s="10" t="n">
+      <c r="E81" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F81" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="F81" s="11" t="inlineStr">
+      <c r="G81" s="11" t="inlineStr">
         <is>
           <t>Pera, ciruela, jazmín, vainilla, cedro. Floral moderno femenino.</t>
         </is>
       </c>
-      <c r="G81" s="12" t="n">
+      <c r="H81" s="12" t="n">
         <v>5800</v>
       </c>
-      <c r="H81" s="13" t="n"/>
-      <c r="I81" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I81" s="13" t="n"/>
       <c r="J81" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K81" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K81" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L81" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.59228.jpg</t>
         </is>
@@ -4379,29 +4784,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E82" s="2" t="n">
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="F82" s="3" t="inlineStr">
+      <c r="G82" s="3" t="inlineStr">
         <is>
           <t>Cactus, rosa, jazmín, sándalo. Verde floral fresco.</t>
         </is>
       </c>
-      <c r="G82" s="4" t="n">
+      <c r="H82" s="4" t="n">
         <v>5500</v>
       </c>
-      <c r="H82" s="5" t="n"/>
-      <c r="I82" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I82" s="5" t="n"/>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K82" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L82" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.25298.jpg</t>
         </is>
@@ -4426,29 +4836,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E83" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F83" s="11" t="inlineStr">
+      <c r="E83" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F83" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G83" s="11" t="inlineStr">
         <is>
           <t>Manzana, camelia, rosa, lirio, bayas silvestres. Americana fresca.</t>
         </is>
       </c>
-      <c r="G83" s="12" t="n">
+      <c r="H83" s="12" t="n">
         <v>4800</v>
       </c>
-      <c r="H83" s="13" t="n"/>
-      <c r="I83" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I83" s="13" t="n"/>
       <c r="J83" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K83" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K83" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L83" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.3016.jpg</t>
         </is>
@@ -4473,29 +4888,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E84" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F84" s="3" t="inlineStr">
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
         <is>
           <t>Pera, vainilla bourbon, habas tonka, flor de sal. Gourmand luminoso.</t>
         </is>
       </c>
-      <c r="G84" s="4" t="n">
+      <c r="H84" s="4" t="n">
         <v>7500</v>
       </c>
-      <c r="H84" s="5" t="n"/>
-      <c r="I84" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I84" s="5" t="n"/>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K84" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L84" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.55786.jpg</t>
         </is>
@@ -4520,29 +4940,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E85" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F85" s="11" t="inlineStr">
+      <c r="E85" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F85" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G85" s="11" t="inlineStr">
         <is>
           <t>Anís, mandarina, rosa, jengibre, vainilla, ámbar. Oriental icónico.</t>
         </is>
       </c>
-      <c r="G85" s="12" t="n">
+      <c r="H85" s="12" t="n">
         <v>7200</v>
       </c>
-      <c r="H85" s="13" t="n"/>
-      <c r="I85" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I85" s="13" t="n"/>
       <c r="J85" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K85" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K85" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L85" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.394.jpg</t>
         </is>
@@ -4567,29 +4992,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E86" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F86" s="3" t="inlineStr">
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
         <is>
           <t>Mandarina, grosella negra, violeta, rosa, haba tonka, almizcle blanco.</t>
         </is>
       </c>
-      <c r="G86" s="4" t="n">
+      <c r="H86" s="4" t="n">
         <v>6800</v>
       </c>
-      <c r="H86" s="5" t="n"/>
-      <c r="I86" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I86" s="5" t="n"/>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K86" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L86" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.72.jpg</t>
         </is>
@@ -4614,29 +5044,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E87" s="10" t="n">
+      <c r="E87" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F87" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="F87" s="11" t="inlineStr">
+      <c r="G87" s="11" t="inlineStr">
         <is>
           <t>Limón, lima, manzana dulce, peonía, vainilla. Frutal floral gourmand.</t>
         </is>
       </c>
-      <c r="G87" s="12" t="n">
+      <c r="H87" s="12" t="n">
         <v>5500</v>
       </c>
-      <c r="H87" s="13" t="n"/>
-      <c r="I87" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I87" s="13" t="n"/>
       <c r="J87" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K87" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K87" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L87" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.147.jpg</t>
         </is>
@@ -4661,29 +5096,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E88" s="2" t="n">
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="F88" s="3" t="inlineStr">
+      <c r="G88" s="3" t="inlineStr">
         <is>
           <t>Pomelo, caramelo, azahar, algodón de azúcar. Frutal dulce joven.</t>
         </is>
       </c>
-      <c r="G88" s="4" t="n">
+      <c r="H88" s="4" t="n">
         <v>5200</v>
       </c>
-      <c r="H88" s="5" t="n"/>
-      <c r="I88" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I88" s="5" t="n"/>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K88" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L88" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.39376.jpg</t>
         </is>
@@ -4708,29 +5148,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E89" s="10" t="n">
+      <c r="E89" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F89" s="10" t="n">
         <v>65</v>
       </c>
-      <c r="F89" s="11" t="inlineStr">
+      <c r="G89" s="11" t="inlineStr">
         <is>
           <t>Bambú, nashi, loto, teca, madreperla. Acuático transparente.</t>
         </is>
       </c>
-      <c r="G89" s="12" t="n">
+      <c r="H89" s="12" t="n">
         <v>5800</v>
       </c>
-      <c r="H89" s="13" t="n"/>
-      <c r="I89" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I89" s="13" t="n"/>
       <c r="J89" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K89" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K89" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L89" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.152.jpg</t>
         </is>
@@ -4755,29 +5200,34 @@
           <t>Mujer</t>
         </is>
       </c>
-      <c r="E90" s="2" t="n">
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="F90" s="3" t="inlineStr">
+      <c r="G90" s="3" t="inlineStr">
         <is>
           <t>Peonía, lichi, freesia, rosa, magnolia, cedro. Floral rosado icónico.</t>
         </is>
       </c>
-      <c r="G90" s="4" t="n">
+      <c r="H90" s="4" t="n">
         <v>9500</v>
       </c>
-      <c r="H90" s="5" t="n"/>
-      <c r="I90" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I90" s="5" t="n"/>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K90" s="3" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L90" s="3" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.1733.jpg</t>
         </is>
@@ -4802,44 +5252,52 @@
           <t>Hombre</t>
         </is>
       </c>
-      <c r="E91" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F91" s="11" t="inlineStr">
+      <c r="E91" s="10" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="F91" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G91" s="11" t="inlineStr">
         <is>
           <t>Mandarina, petitgrain, almíbar, musgo marino. Fresco acuático mineral.</t>
         </is>
       </c>
-      <c r="G91" s="12" t="n">
+      <c r="H91" s="12" t="n">
         <v>6800</v>
       </c>
-      <c r="H91" s="13" t="n"/>
-      <c r="I91" s="10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="I91" s="13" t="n"/>
       <c r="J91" s="10" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K91" s="11" t="inlineStr">
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K91" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L91" s="11" t="inlineStr">
         <is>
           <t>https://fimgs.net/mdimg/perfume/375x500.153.jpg</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="I2:I91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="J2:J91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Hombre,Mujer,Unisex"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Diseñador,Árabe,Nicho"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>